<commit_message>
llm com metade do tempo
</commit_message>
<xml_diff>
--- a/source/out25/relatorio_validacao_gabarito.xlsx
+++ b/source/out25/relatorio_validacao_gabarito.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="120">
   <si>
     <t>idx_df1</t>
   </si>
@@ -61,273 +61,273 @@
     <t>acertou_idx_df2</t>
   </si>
   <si>
+    <t>AVENIDA ANTONIO PIRANGA CENTRO</t>
+  </si>
+  <si>
+    <t>RUA DOS CARIRIS PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>PRACA RUI BARBOSA PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>RUA CAPIBARIBE JARDIM CAMPANARIO</t>
+  </si>
+  <si>
+    <t>AV PIRAPORINHA PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>RUA JOSE BONIFACIO SERRARIA</t>
+  </si>
+  <si>
+    <t>RUA TIRADENTES CENTRO</t>
+  </si>
+  <si>
+    <t>RUA MEM DE SA JARDIM CASA GRANDE</t>
+  </si>
+  <si>
+    <t>AVN SAO JOSE CENTRO</t>
+  </si>
+  <si>
+    <t>RUA SEBASTIAO FERNANDES TOURINHO VIL NOGUEIRA</t>
+  </si>
+  <si>
+    <t>RUA JOSE VICENTE JD INAMAR</t>
+  </si>
+  <si>
+    <t>AV ELDORADO JARDIM RUYCE</t>
+  </si>
+  <si>
+    <t>RUA PRUDENTE DE MORAIS JARDIM CASA GRANDE</t>
+  </si>
+  <si>
+    <t>AV LICO MAIA SERRARIA</t>
+  </si>
+  <si>
+    <t>RUA CARAMURU VL CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA NELSON RODRIGUES VL CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA SANTO AMARO CENTRO</t>
+  </si>
+  <si>
+    <t>RUA SAO JORGE CENTRO</t>
+  </si>
+  <si>
+    <t>ANTONIO PIRANGA CENTRO</t>
+  </si>
+  <si>
+    <t>AVENIDA NOSSA SENHORA DOS NAVEGANTES ELDORADO</t>
+  </si>
+  <si>
+    <t>RUA GRACIOSA CENTRO</t>
+  </si>
+  <si>
+    <t>AV ANTONIO PIRANGA CENTRO</t>
+  </si>
+  <si>
+    <t>AV NOSSA SENHORA DOS NAVEGANTES ELDORADO</t>
+  </si>
+  <si>
+    <t>RUA COIMBRA CENTRO</t>
+  </si>
+  <si>
+    <t>RUA 22 DE ABRIL JD CANHEMA</t>
+  </si>
+  <si>
+    <t>AVN PRESIDENTE JUSCELINO PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>RUA BOROROS CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA ODETE AMARAL DE OLIVEIRA PRQ REAL</t>
+  </si>
+  <si>
+    <t>RUA JAVARI JD PAINEIRAS</t>
+  </si>
+  <si>
+    <t>RUA JAVARI JARDIM PAINEIRAS</t>
+  </si>
+  <si>
+    <t>RUA MANOEL DA NOBREGA VL CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA DAS AMEIXEIRAS JD ABC</t>
+  </si>
+  <si>
+    <t>RUA ITALIA JARDIM DAS NACOES</t>
+  </si>
+  <si>
+    <t>RUA SERRA DE MARACUJA PARQUE REID</t>
+  </si>
+  <si>
+    <t>RUA BARAO DE IGUAPE VIL SAO JOSE</t>
+  </si>
+  <si>
+    <t>AVENIDA AFRANIO PEIXOTO VILA PAULINA</t>
+  </si>
+  <si>
+    <t>RUA MOACIAR GOULART CUNHA CALDAS CENTRO</t>
+  </si>
+  <si>
     <t>AVENIDA SINESIO PEREIRA CAMPANARIO</t>
   </si>
   <si>
-    <t>AVENIDA ANTONIO PIRANGA CENTRO</t>
-  </si>
-  <si>
-    <t>RUA DOS CARIRIS PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>PRACA RUI BARBOSA PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA CAPIBARIBE JARDIM CAMPANARIO</t>
-  </si>
-  <si>
-    <t>AV PIRAPORINHA PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA JOSE BONIFACIO SERRARIA</t>
-  </si>
-  <si>
-    <t>RUA TIRADENTES CENTRO</t>
-  </si>
-  <si>
-    <t>RUA MEM DE SA JARDIM CASA GRANDE</t>
-  </si>
-  <si>
-    <t>AVN SAO JOSE CENTRO</t>
-  </si>
-  <si>
-    <t>RUA SEBASTIAO FERNANDES TOURINHO VIL NOGUEIRA</t>
-  </si>
-  <si>
-    <t>RUA JOSE VICENTE JD INAMAR</t>
-  </si>
-  <si>
-    <t>AV ELDORADO JARDIM RUYCE</t>
-  </si>
-  <si>
-    <t>RUA PRUDENTE DE MORAIS JARDIM CASA GRANDE</t>
-  </si>
-  <si>
-    <t>AV LICO MAIA SERRARIA</t>
-  </si>
-  <si>
-    <t>RUA CARAMURU VL CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA NELSON RODRIGUES VL CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA SANTO AMARO CENTRO</t>
-  </si>
-  <si>
-    <t>RUA SAO JORGE CENTRO</t>
-  </si>
-  <si>
-    <t>ANTONIO PIRANGA CENTRO</t>
-  </si>
-  <si>
-    <t>AVENIDA NOSSA SENHORA DOS NAVEGANTES ELDORADO</t>
-  </si>
-  <si>
-    <t>RUA GRACIOSA CENTRO</t>
-  </si>
-  <si>
-    <t>AV ANTONIO PIRANGA CENTRO</t>
-  </si>
-  <si>
-    <t>AV NOSSA SENHORA DOS NAVEGANTES ELDORADO</t>
-  </si>
-  <si>
-    <t>RUA COIMBRA CENTRO</t>
-  </si>
-  <si>
-    <t>RUA 22 DE ABRIL JD CANHEMA</t>
-  </si>
-  <si>
-    <t>AVN PRESIDENTE JUSCELINO PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA BOROROS CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA JAVARI JD PAINEIRAS</t>
-  </si>
-  <si>
-    <t>RUA JAVARI JARDIM PAINEIRAS</t>
-  </si>
-  <si>
-    <t>RUA MANOEL DA NOBREGA VL CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA DAS AMEIXEIRAS JD ABC</t>
-  </si>
-  <si>
-    <t>RUA BARAO DE IGUAPE VIL SAO JOSE</t>
-  </si>
-  <si>
-    <t>RUA ITALIA JARDIM DAS NACOES</t>
-  </si>
-  <si>
-    <t>RUA ODETE AMARAL DE OLIVEIRA PRQ REAL</t>
-  </si>
-  <si>
-    <t>RUA SERRA DE MARACUJA PARQUE REID</t>
-  </si>
-  <si>
-    <t>AVENIDA AFRANIO PEIXOTO VILA PAULINA</t>
-  </si>
-  <si>
-    <t>RUA MOACIAR GOULART CUNHA CALDAS CENTRO</t>
+    <t>centro</t>
+  </si>
+  <si>
+    <t>piraporinha</t>
+  </si>
+  <si>
+    <t>jardim campanario</t>
+  </si>
+  <si>
+    <t>serraria</t>
+  </si>
+  <si>
+    <t>jardim casa grande</t>
+  </si>
+  <si>
+    <t>vila nogueira</t>
+  </si>
+  <si>
+    <t>jardim inamar</t>
+  </si>
+  <si>
+    <t>jardim ruyce</t>
+  </si>
+  <si>
+    <t>vila conceicao</t>
+  </si>
+  <si>
+    <t>eldorado</t>
+  </si>
+  <si>
+    <t>jardim canhema</t>
+  </si>
+  <si>
+    <t>conceicao</t>
+  </si>
+  <si>
+    <t>parque real</t>
+  </si>
+  <si>
+    <t>jardim paineiras</t>
+  </si>
+  <si>
+    <t>jardim abc</t>
+  </si>
+  <si>
+    <t>jardim das nacoes</t>
+  </si>
+  <si>
+    <t>parque reid</t>
+  </si>
+  <si>
+    <t>vila sao jose</t>
+  </si>
+  <si>
+    <t>vila paulina</t>
   </si>
   <si>
     <t>campanario</t>
   </si>
   <si>
-    <t>centro</t>
-  </si>
-  <si>
-    <t>piraporinha</t>
-  </si>
-  <si>
-    <t>jardim campanario</t>
-  </si>
-  <si>
-    <t>serraria</t>
-  </si>
-  <si>
-    <t>jardim casa grande</t>
-  </si>
-  <si>
-    <t>vila nogueira</t>
-  </si>
-  <si>
-    <t>jardim inamar</t>
-  </si>
-  <si>
-    <t>jardim ruyce</t>
-  </si>
-  <si>
-    <t>vila conceicao</t>
-  </si>
-  <si>
-    <t>eldorado</t>
-  </si>
-  <si>
-    <t>jardim canhema</t>
-  </si>
-  <si>
-    <t>conceicao</t>
-  </si>
-  <si>
-    <t>jardim paineiras</t>
-  </si>
-  <si>
-    <t>jardim abc</t>
-  </si>
-  <si>
-    <t>vila sao jose</t>
-  </si>
-  <si>
-    <t>jardim das nacoes</t>
-  </si>
-  <si>
-    <t>parque real</t>
-  </si>
-  <si>
-    <t>parque reid</t>
-  </si>
-  <si>
-    <t>vila paulina</t>
+    <t>AVENIDA  ANTONIO PIRANGA CENTRO</t>
+  </si>
+  <si>
+    <t>RUA  DOS CARIRIS PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>PRACA  RUI BARBOSA PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>RUA  CAPIBARIBE CAMPANARIO</t>
+  </si>
+  <si>
+    <t>AVENIDA  PIRAPORINHA PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>RUA  JOSE BONIFACIO SERRARIA</t>
+  </si>
+  <si>
+    <t>RUA  TIRADENTES CENTRO</t>
+  </si>
+  <si>
+    <t>RUA  MEM DE SA CASA GRANDE</t>
+  </si>
+  <si>
+    <t>AVENIDA SAO JOSE CENTRO</t>
+  </si>
+  <si>
+    <t>RUA  SEBASTIAO FERNANDES TOURINHO VILA NOGUEIRA</t>
+  </si>
+  <si>
+    <t>RUA  JOSE VICENTE INAMAR</t>
+  </si>
+  <si>
+    <t>AVENIDA  ELDORADO JARDIM RUYCE</t>
+  </si>
+  <si>
+    <t>RUA  PRUDENTE DE MORAIS CASA GRANDE</t>
+  </si>
+  <si>
+    <t>AVENIDA  LICO MAIA SERRARIA</t>
+  </si>
+  <si>
+    <t>RUA  CARAMURU CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA  NELSON RODRIGUES CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA  GRACIOSA CENTRO</t>
+  </si>
+  <si>
+    <t>RUA  COIMBRA CENTRO</t>
+  </si>
+  <si>
+    <t>RUA  VINTE E DOIS DE ABRIL CANHEMA</t>
+  </si>
+  <si>
+    <t>AVENIDA PRESIDENTE JUSCELINO PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>RUA  BOROROS SERRARIA</t>
+  </si>
+  <si>
+    <t>RUA  ODETE AMARAL DE OLIVEIRA CONCEICAO</t>
+  </si>
+  <si>
+    <t>RUA  JAVARI TABOAO</t>
+  </si>
+  <si>
+    <t>RUA  MANOEL DA NOBREGA CENTRO</t>
+  </si>
+  <si>
+    <t>AVENIDA  DAS AMEIXEIRAS TABOAO</t>
+  </si>
+  <si>
+    <t>RUA  ITALIA TABOAO</t>
+  </si>
+  <si>
+    <t>RUA  SERRA DE MARACUJA CENTRO</t>
+  </si>
+  <si>
+    <t>RUA BARAO DE IGUAPE PIRAPORINHA</t>
+  </si>
+  <si>
+    <t>AVENIDA  AFRANIO PEIXOTO ELDORADO</t>
+  </si>
+  <si>
+    <t>RUA  MOACYR GOULART CUNHA CALDAS CONCEICAO</t>
   </si>
   <si>
     <t>AVENIDA  SYNESIO PEREIRA CAMPANARIO</t>
   </si>
   <si>
-    <t>AVENIDA  ANTONIO PIRANGA CENTRO</t>
-  </si>
-  <si>
-    <t>RUA  DOS CARIRIS PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>PRACA  RUI BARBOSA PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA  CAPIBARIBE CAMPANARIO</t>
-  </si>
-  <si>
-    <t>AVENIDA  PIRAPORINHA PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA  JOSE BONIFACIO SERRARIA</t>
-  </si>
-  <si>
-    <t>RUA  TIRADENTES CENTRO</t>
-  </si>
-  <si>
-    <t>RUA  MEM DE SA CASA GRANDE</t>
-  </si>
-  <si>
-    <t>AVENIDA SAO JOSE CENTRO</t>
-  </si>
-  <si>
-    <t>RUA  SEBASTIAO FERNANDES TOURINHO VILA NOGUEIRA</t>
-  </si>
-  <si>
-    <t>RUA  JOSE VICENTE INAMAR</t>
-  </si>
-  <si>
-    <t>AVENIDA  ELDORADO JARDIM RUYCE</t>
-  </si>
-  <si>
-    <t>RUA  PRUDENTE DE MORAIS CASA GRANDE</t>
-  </si>
-  <si>
-    <t>AVENIDA  LICO MAIA SERRARIA</t>
-  </si>
-  <si>
-    <t>RUA  CARAMURU CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA  NELSON RODRIGUES CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA  GRACIOSA CENTRO</t>
-  </si>
-  <si>
-    <t>RUA  COIMBRA CENTRO</t>
-  </si>
-  <si>
-    <t>RUA  VINTE E DOIS DE ABRIL CANHEMA</t>
-  </si>
-  <si>
-    <t>AVENIDA PRESIDENTE JUSCELINO PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA  BOROROS SERRARIA</t>
-  </si>
-  <si>
-    <t>RUA  JAVARI TABOAO</t>
-  </si>
-  <si>
-    <t>RUA  MANOEL DA NOBREGA CENTRO</t>
-  </si>
-  <si>
-    <t>AVENIDA  DAS AMEIXEIRAS TABOAO</t>
-  </si>
-  <si>
-    <t>RUA BARAO DE IGUAPE PIRAPORINHA</t>
-  </si>
-  <si>
-    <t>RUA  ITALIA TABOAO</t>
-  </si>
-  <si>
-    <t>RUA  ODETE AMARAL DE OLIVEIRA CONCEICAO</t>
-  </si>
-  <si>
-    <t>RUA  SERRA DE MARACUJA CENTRO</t>
-  </si>
-  <si>
-    <t>AVENIDA  AFRANIO PEIXOTO ELDORADO</t>
-  </si>
-  <si>
-    <t>RUA  MOACYR GOULART CUNHA CALDAS CONCEICAO</t>
-  </si>
-  <si>
     <t>casa grande</t>
   </si>
   <si>
@@ -338,12 +338,6 @@
   </si>
   <si>
     <t>taboao</t>
-  </si>
-  <si>
-    <t>RUA  LUIS ANTONIO PEREIRA COOPERATIVA</t>
-  </si>
-  <si>
-    <t>COOPERATIVA</t>
   </si>
   <si>
     <t>CENTRO</t>
@@ -789,72 +783,72 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
       </c>
       <c r="C2">
-        <v>27</v>
+        <v>700</v>
       </c>
       <c r="D2" t="s">
         <v>53</v>
       </c>
       <c r="E2">
-        <v>25087</v>
+        <v>50282</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
       <c r="G2">
-        <v>27</v>
+        <v>700</v>
       </c>
       <c r="H2" t="s">
         <v>53</v>
       </c>
       <c r="I2">
-        <v>95.33</v>
+        <v>100</v>
       </c>
       <c r="J2">
-        <v>513300</v>
+        <v>50282</v>
       </c>
       <c r="K2" t="s">
+        <v>73</v>
+      </c>
+      <c r="L2">
+        <v>700</v>
+      </c>
+      <c r="M2" t="s">
         <v>108</v>
       </c>
-      <c r="L2">
-        <v>221</v>
-      </c>
-      <c r="M2" t="s">
-        <v>109</v>
-      </c>
       <c r="N2">
-        <v>64.8</v>
+        <v>100</v>
       </c>
       <c r="O2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>700</v>
+        <v>195</v>
       </c>
       <c r="D3" t="s">
         <v>54</v>
       </c>
       <c r="E3">
-        <v>50282</v>
+        <v>3541</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
       <c r="G3">
-        <v>700</v>
+        <v>195</v>
       </c>
       <c r="H3" t="s">
         <v>54</v>
@@ -863,16 +857,16 @@
         <v>100</v>
       </c>
       <c r="J3">
-        <v>50282</v>
+        <v>3541</v>
       </c>
       <c r="K3" t="s">
         <v>74</v>
       </c>
       <c r="L3">
-        <v>700</v>
+        <v>195</v>
       </c>
       <c r="M3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N3">
         <v>100</v>
@@ -883,43 +877,43 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
       </c>
       <c r="C4">
-        <v>195</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E4">
-        <v>3541</v>
+        <v>160130</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
       <c r="G4">
-        <v>195</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I4">
         <v>100</v>
       </c>
       <c r="J4">
-        <v>3541</v>
+        <v>160130</v>
       </c>
       <c r="K4" t="s">
         <v>75</v>
       </c>
       <c r="L4">
-        <v>195</v>
+        <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="N4">
         <v>100</v>
@@ -930,43 +924,43 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
       </c>
       <c r="C5">
-        <v>27</v>
+        <v>193</v>
       </c>
       <c r="D5" t="s">
         <v>55</v>
       </c>
       <c r="E5">
-        <v>160130</v>
+        <v>115200</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
       <c r="G5">
-        <v>27</v>
+        <v>193</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="I5">
         <v>100</v>
       </c>
       <c r="J5">
-        <v>160130</v>
+        <v>115200</v>
       </c>
       <c r="K5" t="s">
         <v>76</v>
       </c>
       <c r="L5">
-        <v>27</v>
+        <v>193</v>
       </c>
       <c r="M5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N5">
         <v>100</v>
@@ -977,43 +971,43 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="C6">
-        <v>193</v>
+        <v>1682</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E6">
-        <v>115200</v>
+        <v>30100</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
       <c r="G6">
-        <v>193</v>
+        <v>1682</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I6">
         <v>100</v>
       </c>
       <c r="J6">
-        <v>115200</v>
+        <v>30100</v>
       </c>
       <c r="K6" t="s">
         <v>77</v>
       </c>
       <c r="L6">
-        <v>193</v>
+        <v>1682</v>
       </c>
       <c r="M6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="N6">
         <v>100</v>
@@ -1024,40 +1018,40 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
       </c>
       <c r="C7">
-        <v>1682</v>
+        <v>1641</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E7">
-        <v>30100</v>
+        <v>74232</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
       <c r="G7">
-        <v>1682</v>
+        <v>1641</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I7">
         <v>100</v>
       </c>
       <c r="J7">
-        <v>30100</v>
+        <v>74232</v>
       </c>
       <c r="K7" t="s">
         <v>78</v>
       </c>
       <c r="L7">
-        <v>1682</v>
+        <v>1641</v>
       </c>
       <c r="M7" t="s">
         <v>111</v>
@@ -1071,43 +1065,43 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
       </c>
       <c r="C8">
-        <v>1641</v>
+        <v>100</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E8">
-        <v>74232</v>
+        <v>39595</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
       <c r="G8">
-        <v>1641</v>
+        <v>100</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I8">
         <v>100</v>
       </c>
       <c r="J8">
-        <v>74232</v>
+        <v>39595</v>
       </c>
       <c r="K8" t="s">
         <v>79</v>
       </c>
       <c r="L8">
-        <v>1641</v>
+        <v>100</v>
       </c>
       <c r="M8" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="N8">
         <v>100</v>
@@ -1118,43 +1112,43 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
       </c>
       <c r="C9">
-        <v>100</v>
+        <v>280</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E9">
-        <v>39595</v>
+        <v>172305</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
       <c r="G9">
-        <v>100</v>
+        <v>280</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="I9">
         <v>100</v>
       </c>
       <c r="J9">
-        <v>39595</v>
+        <v>172305</v>
       </c>
       <c r="K9" t="s">
         <v>80</v>
       </c>
       <c r="L9">
-        <v>100</v>
+        <v>280</v>
       </c>
       <c r="M9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N9">
         <v>100</v>
@@ -1165,43 +1159,43 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
       </c>
       <c r="C10">
-        <v>280</v>
+        <v>472</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E10">
-        <v>172305</v>
+        <v>89141</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
       <c r="G10">
-        <v>280</v>
+        <v>472</v>
       </c>
       <c r="H10" t="s">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="I10">
         <v>100</v>
       </c>
       <c r="J10">
-        <v>172305</v>
+        <v>89141</v>
       </c>
       <c r="K10" t="s">
         <v>81</v>
       </c>
       <c r="L10">
-        <v>280</v>
+        <v>472</v>
       </c>
       <c r="M10" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="N10">
         <v>100</v>
@@ -1212,43 +1206,43 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
         <v>24</v>
       </c>
       <c r="C11">
-        <v>472</v>
+        <v>285</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E11">
-        <v>89141</v>
+        <v>27959</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
       <c r="G11">
-        <v>472</v>
+        <v>285</v>
       </c>
       <c r="H11" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I11">
         <v>100</v>
       </c>
       <c r="J11">
-        <v>89141</v>
+        <v>27959</v>
       </c>
       <c r="K11" t="s">
         <v>82</v>
       </c>
       <c r="L11">
-        <v>472</v>
+        <v>285</v>
       </c>
       <c r="M11" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="N11">
         <v>100</v>
@@ -1259,43 +1253,43 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
         <v>25</v>
       </c>
       <c r="C12">
-        <v>285</v>
+        <v>122</v>
       </c>
       <c r="D12" t="s">
         <v>59</v>
       </c>
       <c r="E12">
-        <v>27959</v>
+        <v>99539</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
       <c r="G12">
-        <v>285</v>
+        <v>122</v>
       </c>
       <c r="H12" t="s">
-        <v>59</v>
+        <v>105</v>
       </c>
       <c r="I12">
         <v>100</v>
       </c>
       <c r="J12">
-        <v>27959</v>
+        <v>99539</v>
       </c>
       <c r="K12" t="s">
         <v>83</v>
       </c>
       <c r="L12">
-        <v>285</v>
+        <v>122</v>
       </c>
       <c r="M12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="N12">
         <v>100</v>
@@ -1306,43 +1300,43 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
       </c>
       <c r="C13">
-        <v>122</v>
+        <v>817</v>
       </c>
       <c r="D13" t="s">
         <v>60</v>
       </c>
       <c r="E13">
-        <v>99539</v>
+        <v>98493</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
       <c r="G13">
-        <v>122</v>
+        <v>817</v>
       </c>
       <c r="H13" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="I13">
         <v>100</v>
       </c>
       <c r="J13">
-        <v>99539</v>
+        <v>98493</v>
       </c>
       <c r="K13" t="s">
         <v>84</v>
       </c>
       <c r="L13">
-        <v>122</v>
+        <v>817</v>
       </c>
       <c r="M13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N13">
         <v>100</v>
@@ -1353,43 +1347,43 @@
     </row>
     <row r="14" spans="1:15">
       <c r="A14">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
         <v>27</v>
       </c>
       <c r="C14">
-        <v>817</v>
+        <v>300</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E14">
-        <v>98493</v>
+        <v>139970</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
       <c r="G14">
-        <v>817</v>
+        <v>300</v>
       </c>
       <c r="H14" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="I14">
         <v>100</v>
       </c>
       <c r="J14">
-        <v>98493</v>
+        <v>139970</v>
       </c>
       <c r="K14" t="s">
         <v>85</v>
       </c>
       <c r="L14">
-        <v>817</v>
+        <v>300</v>
       </c>
       <c r="M14" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="N14">
         <v>100</v>
@@ -1400,43 +1394,43 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>28</v>
       </c>
       <c r="C15">
-        <v>300</v>
+        <v>803</v>
       </c>
       <c r="D15" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E15">
-        <v>139970</v>
+        <v>11343</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
       <c r="G15">
-        <v>300</v>
+        <v>803</v>
       </c>
       <c r="H15" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="I15">
         <v>100</v>
       </c>
       <c r="J15">
-        <v>139970</v>
+        <v>11343</v>
       </c>
       <c r="K15" t="s">
         <v>86</v>
       </c>
       <c r="L15">
-        <v>300</v>
+        <v>803</v>
       </c>
       <c r="M15" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="N15">
         <v>100</v>
@@ -1447,43 +1441,43 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
       </c>
       <c r="C16">
-        <v>803</v>
+        <v>1255</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E16">
-        <v>11343</v>
+        <v>131520</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
       <c r="G16">
-        <v>803</v>
+        <v>1255</v>
       </c>
       <c r="H16" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="I16">
         <v>100</v>
       </c>
       <c r="J16">
-        <v>11343</v>
+        <v>131520</v>
       </c>
       <c r="K16" t="s">
         <v>87</v>
       </c>
       <c r="L16">
-        <v>803</v>
+        <v>1255</v>
       </c>
       <c r="M16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N16">
         <v>100</v>
@@ -1494,43 +1488,43 @@
     </row>
     <row r="17" spans="1:15">
       <c r="A17">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C17">
-        <v>1255</v>
+        <v>700</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E17">
-        <v>131520</v>
+        <v>50282</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="G17">
-        <v>1255</v>
+        <v>700</v>
       </c>
       <c r="H17" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="I17">
         <v>100</v>
       </c>
       <c r="J17">
-        <v>131520</v>
+        <v>50282</v>
       </c>
       <c r="K17" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="L17">
-        <v>1255</v>
+        <v>700</v>
       </c>
       <c r="M17" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="N17">
         <v>100</v>
@@ -1541,43 +1535,43 @@
     </row>
     <row r="18" spans="1:15">
       <c r="A18">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C18">
-        <v>700</v>
+        <v>191</v>
       </c>
       <c r="D18" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E18">
-        <v>50282</v>
+        <v>67716</v>
       </c>
       <c r="F18" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="G18">
-        <v>700</v>
+        <v>191</v>
       </c>
       <c r="H18" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="I18">
         <v>100</v>
       </c>
       <c r="J18">
-        <v>50282</v>
+        <v>67716</v>
       </c>
       <c r="K18" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="L18">
-        <v>700</v>
+        <v>191</v>
       </c>
       <c r="M18" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="N18">
         <v>100</v>
@@ -1588,43 +1582,43 @@
     </row>
     <row r="19" spans="1:15">
       <c r="A19">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" t="s">
         <v>31</v>
       </c>
       <c r="C19">
-        <v>191</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E19">
-        <v>67716</v>
+        <v>112213</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="G19">
-        <v>191</v>
+        <v>92</v>
       </c>
       <c r="H19" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="I19">
         <v>100</v>
       </c>
       <c r="J19">
-        <v>67716</v>
+        <v>112213</v>
       </c>
       <c r="K19" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="L19">
-        <v>191</v>
+        <v>92</v>
       </c>
       <c r="M19" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="N19">
         <v>100</v>
@@ -1635,43 +1629,43 @@
     </row>
     <row r="20" spans="1:15">
       <c r="A20">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="C20">
-        <v>92</v>
+        <v>556</v>
       </c>
       <c r="D20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E20">
-        <v>112213</v>
+        <v>61402</v>
       </c>
       <c r="F20" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="G20">
-        <v>92</v>
+        <v>556</v>
       </c>
       <c r="H20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I20">
         <v>100</v>
       </c>
       <c r="J20">
-        <v>112213</v>
+        <v>61402</v>
       </c>
       <c r="K20" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="L20">
-        <v>92</v>
+        <v>556</v>
       </c>
       <c r="M20" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N20">
         <v>100</v>
@@ -1682,43 +1676,43 @@
     </row>
     <row r="21" spans="1:15">
       <c r="A21">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="C21">
-        <v>556</v>
+        <v>98</v>
       </c>
       <c r="D21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E21">
-        <v>61402</v>
+        <v>28001</v>
       </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="G21">
-        <v>556</v>
+        <v>98</v>
       </c>
       <c r="H21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I21">
         <v>100</v>
       </c>
       <c r="J21">
-        <v>61402</v>
+        <v>28001</v>
       </c>
       <c r="K21" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="L21">
-        <v>556</v>
+        <v>98</v>
       </c>
       <c r="M21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N21">
         <v>100</v>
@@ -1729,43 +1723,43 @@
     </row>
     <row r="22" spans="1:15">
       <c r="A22">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
         <v>33</v>
       </c>
       <c r="C22">
-        <v>98</v>
+        <v>556</v>
       </c>
       <c r="D22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E22">
-        <v>28001</v>
+        <v>61402</v>
       </c>
       <c r="F22" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="G22">
-        <v>98</v>
+        <v>556</v>
       </c>
       <c r="H22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I22">
         <v>100</v>
       </c>
       <c r="J22">
-        <v>28001</v>
+        <v>61402</v>
       </c>
       <c r="K22" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="L22">
-        <v>98</v>
+        <v>556</v>
       </c>
       <c r="M22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N22">
         <v>100</v>
@@ -1776,43 +1770,43 @@
     </row>
     <row r="23" spans="1:15">
       <c r="A23">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B23" t="s">
         <v>34</v>
       </c>
       <c r="C23">
-        <v>556</v>
+        <v>332</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E23">
-        <v>61402</v>
+        <v>938</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="G23">
-        <v>556</v>
+        <v>332</v>
       </c>
       <c r="H23" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I23">
         <v>100</v>
       </c>
       <c r="J23">
-        <v>61402</v>
+        <v>938</v>
       </c>
       <c r="K23" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="L23">
-        <v>556</v>
+        <v>332</v>
       </c>
       <c r="M23" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="N23">
         <v>100</v>
@@ -1823,43 +1817,40 @@
     </row>
     <row r="24" spans="1:15">
       <c r="A24">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
         <v>35</v>
       </c>
-      <c r="C24">
-        <v>332</v>
-      </c>
       <c r="D24" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E24">
-        <v>938</v>
+        <v>15506</v>
       </c>
       <c r="F24" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="G24">
-        <v>332</v>
+        <v>187</v>
       </c>
       <c r="H24" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I24">
         <v>100</v>
       </c>
       <c r="J24">
-        <v>938</v>
+        <v>15506</v>
       </c>
       <c r="K24" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="L24">
-        <v>332</v>
+        <v>187</v>
       </c>
       <c r="M24" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="N24">
         <v>100</v>
@@ -1870,43 +1861,46 @@
     </row>
     <row r="25" spans="1:15">
       <c r="A25">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="B25" t="s">
         <v>36</v>
       </c>
+      <c r="C25">
+        <v>614</v>
+      </c>
       <c r="D25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E25">
-        <v>15506</v>
+        <v>107930</v>
       </c>
       <c r="F25" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="G25">
-        <v>187</v>
+        <v>615</v>
       </c>
       <c r="H25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I25">
-        <v>100</v>
+        <v>99.97</v>
       </c>
       <c r="J25">
-        <v>15506</v>
+        <v>107930</v>
       </c>
       <c r="K25" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="L25">
-        <v>187</v>
+        <v>615</v>
       </c>
       <c r="M25" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N25">
-        <v>100</v>
+        <v>99.97</v>
       </c>
       <c r="O25" t="b">
         <v>1</v>
@@ -1914,28 +1908,28 @@
     </row>
     <row r="26" spans="1:15">
       <c r="A26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26">
         <v>614</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E26">
         <v>107930</v>
       </c>
       <c r="F26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G26">
         <v>615</v>
       </c>
       <c r="H26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I26">
         <v>99.97</v>
@@ -1944,13 +1938,13 @@
         <v>107930</v>
       </c>
       <c r="K26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L26">
         <v>615</v>
       </c>
       <c r="M26" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N26">
         <v>99.97</v>
@@ -1961,46 +1955,46 @@
     </row>
     <row r="27" spans="1:15">
       <c r="A27">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B27" t="s">
         <v>37</v>
       </c>
       <c r="C27">
-        <v>614</v>
+        <v>288</v>
       </c>
       <c r="D27" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E27">
-        <v>107930</v>
+        <v>43091</v>
       </c>
       <c r="F27" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="G27">
-        <v>615</v>
+        <v>289</v>
       </c>
       <c r="H27" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I27">
-        <v>99.97</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="J27">
-        <v>107930</v>
+        <v>43091</v>
       </c>
       <c r="K27" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="L27">
-        <v>615</v>
+        <v>289</v>
       </c>
       <c r="M27" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="N27">
-        <v>99.97</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="O27" t="b">
         <v>1</v>
@@ -2008,46 +2002,46 @@
     </row>
     <row r="28" spans="1:15">
       <c r="A28">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
       </c>
       <c r="C28">
-        <v>288</v>
+        <v>760</v>
       </c>
       <c r="D28" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E28">
-        <v>43091</v>
+        <v>43728</v>
       </c>
       <c r="F28" t="s">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="G28">
-        <v>289</v>
+        <v>763</v>
       </c>
       <c r="H28" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I28">
-        <v>99.93000000000001</v>
+        <v>99.92</v>
       </c>
       <c r="J28">
-        <v>43091</v>
+        <v>43728</v>
       </c>
       <c r="K28" t="s">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="L28">
-        <v>289</v>
+        <v>763</v>
       </c>
       <c r="M28" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="N28">
-        <v>99.93000000000001</v>
+        <v>99.92</v>
       </c>
       <c r="O28" t="b">
         <v>1</v>
@@ -2055,46 +2049,46 @@
     </row>
     <row r="29" spans="1:15">
       <c r="A29">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
       </c>
       <c r="C29">
-        <v>760</v>
+        <v>113</v>
       </c>
       <c r="D29" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E29">
-        <v>43728</v>
+        <v>179141</v>
       </c>
       <c r="F29" t="s">
         <v>91</v>
       </c>
       <c r="G29">
-        <v>763</v>
+        <v>108</v>
       </c>
       <c r="H29" t="s">
-        <v>54</v>
+        <v>106</v>
       </c>
       <c r="I29">
-        <v>99.92</v>
+        <v>99.12</v>
       </c>
       <c r="J29">
-        <v>43728</v>
+        <v>179141</v>
       </c>
       <c r="K29" t="s">
         <v>91</v>
       </c>
       <c r="L29">
-        <v>763</v>
+        <v>108</v>
       </c>
       <c r="M29" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N29">
-        <v>99.92</v>
+        <v>99.12</v>
       </c>
       <c r="O29" t="b">
         <v>1</v>
@@ -2102,46 +2096,46 @@
     </row>
     <row r="30" spans="1:15">
       <c r="A30">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
       </c>
       <c r="C30">
-        <v>113</v>
+        <v>759</v>
       </c>
       <c r="D30" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E30">
-        <v>179141</v>
+        <v>128655</v>
       </c>
       <c r="F30" t="s">
         <v>92</v>
       </c>
       <c r="G30">
-        <v>108</v>
+        <v>834</v>
       </c>
       <c r="H30" t="s">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="I30">
-        <v>99.12</v>
+        <v>98.2</v>
       </c>
       <c r="J30">
-        <v>179141</v>
+        <v>128655</v>
       </c>
       <c r="K30" t="s">
         <v>92</v>
       </c>
       <c r="L30">
-        <v>108</v>
+        <v>834</v>
       </c>
       <c r="M30" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="N30">
-        <v>99.12</v>
+        <v>98.2</v>
       </c>
       <c r="O30" t="b">
         <v>1</v>
@@ -2149,46 +2143,46 @@
     </row>
     <row r="31" spans="1:15">
       <c r="A31">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B31" t="s">
         <v>41</v>
       </c>
       <c r="C31">
-        <v>759</v>
+        <v>80</v>
       </c>
       <c r="D31" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="E31">
-        <v>128655</v>
+        <v>82323</v>
       </c>
       <c r="F31" t="s">
         <v>93</v>
       </c>
       <c r="G31">
-        <v>834</v>
+        <v>80</v>
       </c>
       <c r="H31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I31">
-        <v>98.2</v>
+        <v>93.53</v>
       </c>
       <c r="J31">
-        <v>128655</v>
+        <v>82323</v>
       </c>
       <c r="K31" t="s">
         <v>93</v>
       </c>
       <c r="L31">
-        <v>834</v>
+        <v>80</v>
       </c>
       <c r="M31" t="s">
         <v>111</v>
       </c>
       <c r="N31">
-        <v>98.2</v>
+        <v>92.34</v>
       </c>
       <c r="O31" t="b">
         <v>1</v>
@@ -2196,46 +2190,46 @@
     </row>
     <row r="32" spans="1:15">
       <c r="A32">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="B32" t="s">
         <v>42</v>
       </c>
       <c r="C32">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="D32" t="s">
         <v>65</v>
       </c>
       <c r="E32">
-        <v>82323</v>
+        <v>168293</v>
       </c>
       <c r="F32" t="s">
         <v>94</v>
       </c>
       <c r="G32">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="H32" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="I32">
-        <v>93.53</v>
+        <v>92</v>
       </c>
       <c r="J32">
-        <v>82323</v>
+        <v>168293</v>
       </c>
       <c r="K32" t="s">
         <v>94</v>
       </c>
       <c r="L32">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="M32" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N32">
-        <v>94.45</v>
+        <v>92.31</v>
       </c>
       <c r="O32" t="b">
         <v>1</v>
@@ -2279,10 +2273,10 @@
         <v>635</v>
       </c>
       <c r="M33" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N33">
-        <v>93.37</v>
+        <v>92.29000000000001</v>
       </c>
       <c r="O33" t="b">
         <v>1</v>
@@ -2326,10 +2320,10 @@
         <v>635</v>
       </c>
       <c r="M34" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N34">
-        <v>93.37</v>
+        <v>92.29000000000001</v>
       </c>
       <c r="O34" t="b">
         <v>1</v>
@@ -2346,7 +2340,7 @@
         <v>605</v>
       </c>
       <c r="D35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E35">
         <v>135351</v>
@@ -2358,7 +2352,7 @@
         <v>605</v>
       </c>
       <c r="H35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I35">
         <v>93</v>
@@ -2373,10 +2367,10 @@
         <v>605</v>
       </c>
       <c r="M35" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N35">
-        <v>93.37</v>
+        <v>92.15000000000001</v>
       </c>
       <c r="O35" t="b">
         <v>1</v>
@@ -2420,10 +2414,10 @@
         <v>679</v>
       </c>
       <c r="M36" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N36">
-        <v>92.95</v>
+        <v>91.67</v>
       </c>
       <c r="O36" t="b">
         <v>1</v>
@@ -2431,46 +2425,46 @@
     </row>
     <row r="37" spans="1:15">
       <c r="A37">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B37" t="s">
         <v>47</v>
       </c>
       <c r="C37">
-        <v>98</v>
+        <v>290</v>
       </c>
       <c r="D37" t="s">
         <v>68</v>
       </c>
       <c r="E37">
-        <v>15269</v>
+        <v>151049</v>
       </c>
       <c r="F37" t="s">
         <v>98</v>
       </c>
       <c r="G37">
-        <v>98</v>
+        <v>290</v>
       </c>
       <c r="H37" t="s">
-        <v>55</v>
+        <v>107</v>
       </c>
       <c r="I37">
-        <v>93.33</v>
+        <v>92.61</v>
       </c>
       <c r="J37">
-        <v>15269</v>
+        <v>151049</v>
       </c>
       <c r="K37" t="s">
         <v>98</v>
       </c>
       <c r="L37">
-        <v>98</v>
+        <v>290</v>
       </c>
       <c r="M37" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="N37">
-        <v>91.95</v>
+        <v>91.17</v>
       </c>
       <c r="O37" t="b">
         <v>1</v>
@@ -2478,46 +2472,46 @@
     </row>
     <row r="38" spans="1:15">
       <c r="A38">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
         <v>48</v>
       </c>
       <c r="C38">
-        <v>290</v>
+        <v>49</v>
       </c>
       <c r="D38" t="s">
         <v>69</v>
       </c>
       <c r="E38">
-        <v>151049</v>
+        <v>69982</v>
       </c>
       <c r="F38" t="s">
         <v>99</v>
       </c>
       <c r="G38">
-        <v>290</v>
+        <v>49</v>
       </c>
       <c r="H38" t="s">
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="I38">
-        <v>92.61</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="J38">
-        <v>151049</v>
+        <v>69982</v>
       </c>
       <c r="K38" t="s">
         <v>99</v>
       </c>
       <c r="L38">
-        <v>290</v>
+        <v>49</v>
       </c>
       <c r="M38" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="N38">
-        <v>91.79000000000001</v>
+        <v>89.83</v>
       </c>
       <c r="O38" t="b">
         <v>1</v>
@@ -2525,46 +2519,46 @@
     </row>
     <row r="39" spans="1:15">
       <c r="A39">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B39" t="s">
         <v>49</v>
       </c>
       <c r="C39">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="D39" t="s">
         <v>70</v>
       </c>
       <c r="E39">
-        <v>168293</v>
+        <v>15269</v>
       </c>
       <c r="F39" t="s">
         <v>100</v>
       </c>
       <c r="G39">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="H39" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="I39">
-        <v>92</v>
+        <v>93.33</v>
       </c>
       <c r="J39">
-        <v>168293</v>
+        <v>15269</v>
       </c>
       <c r="K39" t="s">
         <v>100</v>
       </c>
       <c r="L39">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="M39" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="N39">
-        <v>91.68000000000001</v>
+        <v>89.48</v>
       </c>
       <c r="O39" t="b">
         <v>1</v>
@@ -2572,46 +2566,46 @@
     </row>
     <row r="40" spans="1:15">
       <c r="A40">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="B40" t="s">
         <v>50</v>
       </c>
       <c r="C40">
-        <v>49</v>
+        <v>643</v>
       </c>
       <c r="D40" t="s">
         <v>71</v>
       </c>
       <c r="E40">
-        <v>69982</v>
+        <v>59437</v>
       </c>
       <c r="F40" t="s">
         <v>101</v>
       </c>
       <c r="G40">
-        <v>49</v>
+        <v>599</v>
       </c>
       <c r="H40" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I40">
-        <v>92.34999999999999</v>
+        <v>90.63</v>
       </c>
       <c r="J40">
-        <v>69982</v>
+        <v>59437</v>
       </c>
       <c r="K40" t="s">
         <v>101</v>
       </c>
       <c r="L40">
-        <v>49</v>
+        <v>599</v>
       </c>
       <c r="M40" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="N40">
-        <v>91.38</v>
+        <v>89.12</v>
       </c>
       <c r="O40" t="b">
         <v>1</v>
@@ -2619,46 +2613,46 @@
     </row>
     <row r="41" spans="1:15">
       <c r="A41">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="B41" t="s">
         <v>51</v>
       </c>
       <c r="C41">
-        <v>643</v>
+        <v>111</v>
       </c>
       <c r="D41" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="E41">
-        <v>59437</v>
+        <v>70850</v>
       </c>
       <c r="F41" t="s">
         <v>102</v>
       </c>
       <c r="G41">
-        <v>599</v>
+        <v>111</v>
       </c>
       <c r="H41" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I41">
-        <v>90.63</v>
+        <v>90.18000000000001</v>
       </c>
       <c r="J41">
-        <v>59437</v>
+        <v>70850</v>
       </c>
       <c r="K41" t="s">
         <v>102</v>
       </c>
       <c r="L41">
-        <v>599</v>
+        <v>111</v>
       </c>
       <c r="M41" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="N41">
-        <v>91.06999999999999</v>
+        <v>82.68000000000001</v>
       </c>
       <c r="O41" t="b">
         <v>1</v>
@@ -2666,46 +2660,46 @@
     </row>
     <row r="42" spans="1:15">
       <c r="A42">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="B42" t="s">
         <v>52</v>
       </c>
       <c r="C42">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="D42" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="E42">
-        <v>70850</v>
+        <v>25087</v>
       </c>
       <c r="F42" t="s">
         <v>103</v>
       </c>
       <c r="G42">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="H42" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="I42">
-        <v>90.18000000000001</v>
+        <v>95.33</v>
       </c>
       <c r="J42">
-        <v>70850</v>
+        <v>25087</v>
       </c>
       <c r="K42" t="s">
         <v>103</v>
       </c>
       <c r="L42">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="M42" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="N42">
-        <v>89.09</v>
+        <v>78.27</v>
       </c>
       <c r="O42" t="b">
         <v>1</v>

</xml_diff>